<commit_message>
Refactor preprocessing and add Streamlit deployment
</commit_message>
<xml_diff>
--- a/outputs/data_dictionary_processed.xlsx
+++ b/outputs/data_dictionary_processed.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,7 +490,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>datetime64[us, UTC]</t>
+          <t>datetime64[us]</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -656,12 +656,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>clean_review</t>
+          <t>processed_texts</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>clean_review</t>
+          <t>processed_texts</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -671,29 +671,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cleaned review after normalisation</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>processed_tokens</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>processed_tokens</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Tokenized, lemmatized text with stop words removed</t>
+          <t>Joined tokenized, lemmatized text with stop words removed</t>
         </is>
       </c>
     </row>

</xml_diff>